<commit_message>
Add Min/Max/Fixed Length support
Introduce minLength, maxLength and fixedLength fields across the pipeline: update OrderRow, parse these columns in readExcel (handle empty/null and convert to numbers), and set them on rows (undefined if NaN). Enhance fillItemModal to select Length from the dropdown and handle two modes: Fixed (single length input) and Range (Min/Max inputs), preferring Excel values and falling back to CONFIG defaults when needed. Also update SKILL.md to document the three new fields and include an updated demo2.xlsx.
</commit_message>
<xml_diff>
--- a/demo2.xlsx
+++ b/demo2.xlsx
@@ -466,7 +466,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:K7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -493,62 +493,229 @@
       <c r="H1" t="str">
         <v>Make</v>
       </c>
+      <c r="I1" t="str">
+        <v>Min Length</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Max Length</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Fixed Length</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Hengyang</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>ASMEB36.10-22|ASTM/ASME106-19 B</v>
+        <v>API5L 46th Edition X52 PSL 2</v>
       </c>
       <c r="C2" t="str">
-        <v>NPS 24 STD</v>
-      </c>
-      <c r="D2">
-        <v>3937</v>
+        <v>NPS 34 STD</v>
+      </c>
+      <c r="D2" t="str">
+        <v>710</v>
       </c>
       <c r="E2" t="str">
-        <v>ft</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>DRL</v>
+        <v>Fixed</v>
       </c>
       <c r="G2" t="str">
-        <v>Beveled</v>
+        <v>Plain End Square Cut</v>
       </c>
       <c r="H2" t="str">
-        <v>Seamless</v>
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>60</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Baosteel</v>
+        <v/>
       </c>
       <c r="B3" t="str">
-        <v>ASMEB36.10-22|API5L 46th Edition B PSL 2</v>
+        <v>API5L 46th Edition X52 PSL 2</v>
       </c>
       <c r="C3" t="str">
-        <v>NPS 24 STD</v>
-      </c>
-      <c r="D3">
-        <v>3937</v>
+        <v>NPS 34 STD</v>
+      </c>
+      <c r="D3" t="str">
+        <v>710</v>
       </c>
       <c r="E3" t="str">
-        <v>ft</v>
+        <v/>
       </c>
       <c r="F3" t="str">
         <v>Fixed</v>
       </c>
       <c r="G3" t="str">
-        <v>Beveled</v>
+        <v>Plain End Square Cut</v>
       </c>
       <c r="H3" t="str">
-        <v>ERW</v>
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v>API5L 46th Edition X52 PSL 2</v>
+      </c>
+      <c r="C4" t="str">
+        <v>NPS 34 STD</v>
+      </c>
+      <c r="D4" t="str">
+        <v>710</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v>Fixed</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Plain End Square Cut</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v>API5L 46th Edition X52 PSL 2</v>
+      </c>
+      <c r="C5" t="str">
+        <v>NPS 34 XS</v>
+      </c>
+      <c r="D5" t="str">
+        <v>710</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>Fixed</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Plain End Square Cut</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
+      <c r="B6" t="str">
+        <v>API5L 46th Edition X52 PSL 2</v>
+      </c>
+      <c r="C6" t="str">
+        <v>NPS 34 XS</v>
+      </c>
+      <c r="D6" t="str">
+        <v>710</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>Fixed</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Plain End Square Cut</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v>API5L 46th Edition X52 PSL 2</v>
+      </c>
+      <c r="C7" t="str">
+        <v>NPS 34 XS</v>
+      </c>
+      <c r="D7" t="str">
+        <v>710</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>Fixed</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Plain End Square Cut</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>